<commit_message>
UPdated ReadMe with wiring section. Added new ReadMeAssets files - DR966Manual, updated wiring diagram, and updated BOM.
</commit_message>
<xml_diff>
--- a/ReadMeAssets/DrInfraredHeaterRemoteThermostat_BOM.xlsx
+++ b/ReadMeAssets/DrInfraredHeaterRemoteThermostat_BOM.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d02527ba799f7e57/Desktop/Personel Projects/Shop Heater/Public Repo/Dr-Infrared-Heater-Remote-Thermostat/ReadMe Assets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d02527ba799f7e57/Desktop/Personel Projects/Shop Heater/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="105" documentId="13_ncr:1_{C3E0A6F9-8DAD-4268-B801-F770A0C7E470}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D2E7A27F-CA4A-417F-81CB-854403E51689}"/>
+  <xr:revisionPtr revIDLastSave="185" documentId="13_ncr:1_{C3E0A6F9-8DAD-4268-B801-F770A0C7E470}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B13CF3E-20F6-4825-80EE-0AF5E94DB519}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-90" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="51">
   <si>
     <t>Description</t>
   </si>
@@ -167,7 +167,52 @@
     <t>277-1274-ND</t>
   </si>
   <si>
-    <t>16 gauge wire and proabbly 20 gauge wire</t>
+    <t>B09WB1857W</t>
+  </si>
+  <si>
+    <t>Samsung PRO Endurance 128GB MicroSD Card</t>
+  </si>
+  <si>
+    <t>AWG 10 stranded 600v black wire 25ft</t>
+  </si>
+  <si>
+    <t>AWG 10 stranded 600v green wire 25ft</t>
+  </si>
+  <si>
+    <t>AWG 16 stranded 600v black wire 25ft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AWG 16 stranded 600v green wire 25ft </t>
+  </si>
+  <si>
+    <t>AWG 18 stranded 600v black wire 25ft</t>
+  </si>
+  <si>
+    <t>AWG 18 stranded 600v red wire 25ft</t>
+  </si>
+  <si>
+    <t>8054T29-9154T211</t>
+  </si>
+  <si>
+    <t>8054T29-9154T233</t>
+  </si>
+  <si>
+    <t>8054T26-8054T866</t>
+  </si>
+  <si>
+    <t>8054T25-8054T805</t>
+  </si>
+  <si>
+    <t>8054T25-8054T849</t>
+  </si>
+  <si>
+    <t>AWG 18 stranded 600v yellow wire 25ft</t>
+  </si>
+  <si>
+    <t>B0C56Y6D2W</t>
+  </si>
+  <si>
+    <t>Spade Connector Kit 330pcs</t>
   </si>
 </sst>
 </file>
@@ -288,12 +333,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -302,6 +341,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -320,6 +365,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -585,7 +634,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="60.6328125" customWidth="1"/>
@@ -638,7 +687,7 @@
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="7" t="s">
         <v>13</v>
       </c>
       <c r="C3" s="4" t="s">
@@ -651,37 +700,37 @@
         <v>18</v>
       </c>
       <c r="F3" s="3">
-        <f t="shared" ref="F3:F18" si="0">D3*E3</f>
+        <f t="shared" ref="F3:F20" si="0">D3*E3</f>
         <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>15</v>
+        <v>36</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>35</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="D4" s="2">
         <v>1</v>
       </c>
       <c r="E4" s="3">
-        <v>0.95</v>
+        <v>22.99</v>
       </c>
       <c r="F4" s="3">
         <f t="shared" si="0"/>
-        <v>0.95</v>
+        <v>22.99</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>10</v>
@@ -690,19 +739,19 @@
         <v>1</v>
       </c>
       <c r="E5" s="3">
-        <v>4.5</v>
+        <v>0.95</v>
       </c>
       <c r="F5" s="3">
         <f t="shared" si="0"/>
-        <v>4.5</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>10</v>
@@ -711,145 +760,145 @@
         <v>1</v>
       </c>
       <c r="E6" s="3">
-        <v>9.9499999999999993</v>
+        <v>4.5</v>
       </c>
       <c r="F6" s="3">
         <f t="shared" si="0"/>
-        <v>9.9499999999999993</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C7" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7" s="3">
-        <v>1.93</v>
+        <v>9.9499999999999993</v>
       </c>
       <c r="F7" s="3">
         <f t="shared" si="0"/>
-        <v>3.86</v>
+        <v>9.9499999999999993</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C8" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="8" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="2">
         <v>2</v>
       </c>
       <c r="E8" s="3">
-        <v>2.77</v>
+        <v>1.93</v>
       </c>
       <c r="F8" s="3">
         <f t="shared" si="0"/>
-        <v>5.54</v>
+        <v>3.86</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D9" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E9" s="3">
-        <v>1.22</v>
+        <v>2.77</v>
       </c>
       <c r="F9" s="3">
         <f t="shared" si="0"/>
-        <v>3.66</v>
+        <v>5.54</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D10" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E10" s="3">
-        <v>8.6</v>
+        <v>1.22</v>
       </c>
       <c r="F10" s="3">
         <f t="shared" si="0"/>
-        <v>8.6</v>
+        <v>3.66</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="D11" s="2">
         <v>1</v>
       </c>
       <c r="E11" s="3">
-        <v>10.99</v>
+        <v>8.6</v>
       </c>
       <c r="F11" s="3">
         <f t="shared" si="0"/>
-        <v>10.99</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D12" s="2">
         <v>1</v>
       </c>
       <c r="E12" s="3">
-        <v>4.4800000000000004</v>
+        <v>10.99</v>
       </c>
       <c r="F12" s="3">
         <f t="shared" si="0"/>
-        <v>4.4800000000000004</v>
+        <v>10.99</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>24</v>
@@ -858,102 +907,237 @@
         <v>1</v>
       </c>
       <c r="E13" s="3">
-        <v>6.87</v>
+        <v>4.4800000000000004</v>
       </c>
       <c r="F13" s="3">
         <f t="shared" si="0"/>
-        <v>6.87</v>
+        <v>4.4800000000000004</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="3"/>
+        <v>27</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" s="2">
+        <v>1</v>
+      </c>
+      <c r="E14" s="3">
+        <v>6.87</v>
+      </c>
       <c r="F14" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>6.87</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A15" s="1"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="3"/>
+      <c r="A15" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="2">
+        <v>1</v>
+      </c>
+      <c r="E15" s="3">
+        <v>36.340000000000003</v>
+      </c>
       <c r="F15" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>36.340000000000003</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A16" s="1"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="3"/>
+      <c r="A16" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" s="2">
+        <v>1</v>
+      </c>
+      <c r="E16" s="3">
+        <v>36.340000000000003</v>
+      </c>
       <c r="F16" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>36.340000000000003</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A17" s="1"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="3"/>
+      <c r="A17" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D17" s="2">
+        <v>1</v>
+      </c>
+      <c r="E17" s="3">
+        <v>9.3699999999999992</v>
+      </c>
       <c r="F17" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>9.3699999999999992</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A18" s="1"/>
+      <c r="A18" s="1" t="s">
+        <v>40</v>
+      </c>
       <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="3"/>
+      <c r="C18" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D18" s="2">
+        <v>1</v>
+      </c>
+      <c r="E18" s="3">
+        <v>9.3699999999999992</v>
+      </c>
       <c r="F18" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>9.3699999999999992</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D19" s="2">
+        <v>1</v>
+      </c>
+      <c r="E19" s="3">
+        <v>6.48</v>
+      </c>
+      <c r="F19" s="3">
+        <f t="shared" si="0"/>
+        <v>6.48</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D20" s="2">
+        <v>1</v>
+      </c>
+      <c r="E20" s="3">
+        <v>6.48</v>
+      </c>
+      <c r="F20" s="3">
+        <f t="shared" si="0"/>
+        <v>6.48</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A21" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D21" s="2">
+        <v>1</v>
+      </c>
+      <c r="E21" s="3">
+        <v>6.48</v>
+      </c>
+      <c r="F21" s="3">
+        <f>D21*E21</f>
+        <v>6.48</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D22" s="2">
+        <v>1</v>
+      </c>
+      <c r="E22" s="3">
+        <v>9.19</v>
+      </c>
+      <c r="F22" s="3">
+        <f>D22*E22</f>
+        <v>9.19</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="8">
-        <f>SUM(F2:F18)</f>
-        <v>277.39999999999998</v>
+      <c r="B23" s="10"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="6">
+        <f>SUM(F2:F22)</f>
+        <v>420.44000000000023</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A23:E23"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{7E1BCDF3-976F-4AEC-B6D9-914AB11C8929}"/>
     <hyperlink ref="C3" r:id="rId2" xr:uid="{E9D06958-5AD5-46DF-B69C-3902CC72E8E2}"/>
-    <hyperlink ref="C10" r:id="rId3" xr:uid="{D022BB45-F54B-4EE7-A5EF-F34DA750CE30}"/>
-    <hyperlink ref="C4" r:id="rId4" xr:uid="{DC272C52-B2F4-42A2-A5F6-AD123CB15E40}"/>
-    <hyperlink ref="C5" r:id="rId5" xr:uid="{80FBAC2B-CD83-4D3B-8BCB-0BFF059C9B09}"/>
-    <hyperlink ref="C6" r:id="rId6" xr:uid="{A472254A-DB72-4F80-8E3F-549AE130CAFE}"/>
-    <hyperlink ref="C11" r:id="rId7" xr:uid="{3A26B573-E34D-469A-A519-C54C4E3D42C0}"/>
-    <hyperlink ref="C12" r:id="rId8" xr:uid="{669AE46F-78EB-41F5-A3DF-EAD27728EBA6}"/>
-    <hyperlink ref="C13" r:id="rId9" xr:uid="{4E218C59-F2C4-4892-A27C-5AFA85EDCA52}"/>
-    <hyperlink ref="C9" r:id="rId10" xr:uid="{733216EA-AAEC-4C8C-B3A9-ADA8A4D0B204}"/>
-    <hyperlink ref="C7" r:id="rId11" xr:uid="{AF2110D2-291F-442A-A5E5-57541CFF8277}"/>
-    <hyperlink ref="C8" r:id="rId12" xr:uid="{7A253563-3D9D-46CC-BC1C-DDD198212179}"/>
+    <hyperlink ref="C11" r:id="rId3" xr:uid="{D022BB45-F54B-4EE7-A5EF-F34DA750CE30}"/>
+    <hyperlink ref="C5" r:id="rId4" xr:uid="{DC272C52-B2F4-42A2-A5F6-AD123CB15E40}"/>
+    <hyperlink ref="C6" r:id="rId5" xr:uid="{80FBAC2B-CD83-4D3B-8BCB-0BFF059C9B09}"/>
+    <hyperlink ref="C7" r:id="rId6" xr:uid="{A472254A-DB72-4F80-8E3F-549AE130CAFE}"/>
+    <hyperlink ref="C12" r:id="rId7" xr:uid="{3A26B573-E34D-469A-A519-C54C4E3D42C0}"/>
+    <hyperlink ref="C13" r:id="rId8" xr:uid="{669AE46F-78EB-41F5-A3DF-EAD27728EBA6}"/>
+    <hyperlink ref="C14" r:id="rId9" xr:uid="{4E218C59-F2C4-4892-A27C-5AFA85EDCA52}"/>
+    <hyperlink ref="C10" r:id="rId10" xr:uid="{733216EA-AAEC-4C8C-B3A9-ADA8A4D0B204}"/>
+    <hyperlink ref="C8" r:id="rId11" xr:uid="{AF2110D2-291F-442A-A5E5-57541CFF8277}"/>
+    <hyperlink ref="C9" r:id="rId12" xr:uid="{7A253563-3D9D-46CC-BC1C-DDD198212179}"/>
+    <hyperlink ref="C4" r:id="rId13" xr:uid="{75515651-AB6C-4B0A-AF5B-7323FD66E4AB}"/>
+    <hyperlink ref="C15" r:id="rId14" xr:uid="{9CEEADEB-655B-4EE8-8A65-4DEDCAEC4AAA}"/>
+    <hyperlink ref="C16" r:id="rId15" xr:uid="{BE6FF4D7-E9DE-4C77-BEED-3EE4C1B0FD1E}"/>
+    <hyperlink ref="C17" r:id="rId16" xr:uid="{54E91CA4-70D4-4C93-A3BC-A9525F2082F5}"/>
+    <hyperlink ref="C19" r:id="rId17" xr:uid="{05371DE3-0E3D-4DFB-AB69-689437183BD1}"/>
+    <hyperlink ref="C20" r:id="rId18" xr:uid="{CB12FF0B-0CD6-4EE9-BE97-CC2265FAA037}"/>
+    <hyperlink ref="C22" r:id="rId19" xr:uid="{D38EB2FB-A4F6-4217-AC04-0696B84A21B7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId13"/>
+  <legacyDrawing r:id="rId20"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated readme style and BOM.
</commit_message>
<xml_diff>
--- a/ReadMeAssets/DrInfraredHeaterRemoteThermostat_BOM.xlsx
+++ b/ReadMeAssets/DrInfraredHeaterRemoteThermostat_BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d02527ba799f7e57/Desktop/Personel Projects/Shop Heater/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\talyn\OneDrive\Desktop\Personel Projects\Shop Heater\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="185" documentId="13_ncr:1_{C3E0A6F9-8DAD-4268-B801-F770A0C7E470}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B13CF3E-20F6-4825-80EE-0AF5E94DB519}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1B8D5FE-E632-49E5-B63D-DF10E83858A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-90" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Items" sheetId="1" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="53">
   <si>
     <t>Description</t>
   </si>
@@ -213,6 +213,12 @@
   </si>
   <si>
     <t>Spade Connector Kit 330pcs</t>
+  </si>
+  <si>
+    <t>3D printed Heater Back Mount Plate</t>
+  </si>
+  <si>
+    <t>3D printed temperature probe case</t>
   </si>
 </sst>
 </file>
@@ -365,10 +371,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -634,7 +636,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="60.6328125" customWidth="1"/>
@@ -1100,21 +1102,45 @@
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A23" s="9" t="s">
+      <c r="A23" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B23" s="2"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="2">
+        <v>1</v>
+      </c>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B24" s="2"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="2">
+        <v>1</v>
+      </c>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B23" s="10"/>
-      <c r="C23" s="10"/>
-      <c r="D23" s="10"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="6">
+      <c r="B25" s="10"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="6">
         <f>SUM(F2:F22)</f>
         <v>420.44000000000023</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A25:E25"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{7E1BCDF3-976F-4AEC-B6D9-914AB11C8929}"/>

</xml_diff>

<commit_message>
Updated BOM with screws. Added new image to readMe of temperature probe case. Added temp probe case image.
</commit_message>
<xml_diff>
--- a/ReadMeAssets/DrInfraredHeaterRemoteThermostat_BOM.xlsx
+++ b/ReadMeAssets/DrInfraredHeaterRemoteThermostat_BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\talyn\OneDrive\Desktop\Personel Projects\Shop Heater\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1B8D5FE-E632-49E5-B63D-DF10E83858A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A137902-908A-4BFB-B5F6-04D42BEFF680}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-90" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Items" sheetId="1" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="56">
   <si>
     <t>Description</t>
   </si>
@@ -219,6 +219,15 @@
   </si>
   <si>
     <t>3D printed temperature probe case</t>
+  </si>
+  <si>
+    <t>Menards</t>
+  </si>
+  <si>
+    <t>Probe case screws (#8 X 3/4-Inch Phillips Pan-Head screw)</t>
+  </si>
+  <si>
+    <t>Back mount plate screws (#6 x 1/2-Inch Phillips Pan-Head screw)</t>
   </si>
 </sst>
 </file>
@@ -636,7 +645,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="60.6328125" customWidth="1"/>
@@ -1111,36 +1120,84 @@
         <v>1</v>
       </c>
       <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
+      <c r="F23" s="3">
+        <f t="shared" ref="F23:F26" si="1">D23*E23</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B24" s="2">
+        <v>2337250</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D24" s="2">
+        <v>1</v>
+      </c>
+      <c r="E24" s="3">
+        <v>1.28</v>
+      </c>
+      <c r="F24" s="3">
+        <f t="shared" si="1"/>
+        <v>1.28</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="2"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="2">
-        <v>1</v>
-      </c>
-      <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A25" s="9" t="s">
+      <c r="B25" s="2"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="2">
+        <v>1</v>
+      </c>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B26" s="2">
+        <v>2010225</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D26" s="2">
+        <v>1</v>
+      </c>
+      <c r="E26" s="3">
+        <v>1.19</v>
+      </c>
+      <c r="F26" s="3">
+        <f t="shared" si="1"/>
+        <v>1.19</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B25" s="10"/>
-      <c r="C25" s="10"/>
-      <c r="D25" s="10"/>
-      <c r="E25" s="10"/>
-      <c r="F25" s="6">
+      <c r="B27" s="10"/>
+      <c r="C27" s="10"/>
+      <c r="D27" s="10"/>
+      <c r="E27" s="10"/>
+      <c r="F27" s="6">
         <f>SUM(F2:F22)</f>
         <v>420.44000000000023</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A27:E27"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{7E1BCDF3-976F-4AEC-B6D9-914AB11C8929}"/>
@@ -1162,8 +1219,10 @@
     <hyperlink ref="C19" r:id="rId17" xr:uid="{05371DE3-0E3D-4DFB-AB69-689437183BD1}"/>
     <hyperlink ref="C20" r:id="rId18" xr:uid="{CB12FF0B-0CD6-4EE9-BE97-CC2265FAA037}"/>
     <hyperlink ref="C22" r:id="rId19" xr:uid="{D38EB2FB-A4F6-4217-AC04-0696B84A21B7}"/>
+    <hyperlink ref="C26" r:id="rId20" xr:uid="{552C1563-638D-45A1-AC3A-44E4E9AF22B2}"/>
+    <hyperlink ref="C24" r:id="rId21" xr:uid="{F9C09103-24AD-4BE0-98BE-EAA8979D84BF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId20"/>
+  <legacyDrawing r:id="rId22"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
BOM updated with AWG 20 solid core.
</commit_message>
<xml_diff>
--- a/ReadMeAssets/DrInfraredHeaterRemoteThermostat_BOM.xlsx
+++ b/ReadMeAssets/DrInfraredHeaterRemoteThermostat_BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\talyn\OneDrive\Desktop\Personel Projects\Shop Heater\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A137902-908A-4BFB-B5F6-04D42BEFF680}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EDD81B0-2373-49EA-B874-4BDB67130E9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-90" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="59">
   <si>
     <t>Description</t>
   </si>
@@ -140,12 +140,6 @@
     <t>92005A116</t>
   </si>
   <si>
-    <t>Power Supply Phillips Screw</t>
-  </si>
-  <si>
-    <t>Raspberry Pi and Relay Board Phillips Screw</t>
-  </si>
-  <si>
     <t>92005A052</t>
   </si>
   <si>
@@ -228,6 +222,21 @@
   </si>
   <si>
     <t>Back mount plate screws (#6 x 1/2-Inch Phillips Pan-Head screw)</t>
+  </si>
+  <si>
+    <t>8054T26-8054T02</t>
+  </si>
+  <si>
+    <t>8054T25-8054T861</t>
+  </si>
+  <si>
+    <t>AWG 20 solid 300v yellow wire 25ft</t>
+  </si>
+  <si>
+    <t>Raspberry Pi and Relay Board Phillips Screw (M3 x 0.5mm)</t>
+  </si>
+  <si>
+    <t>Power Supply Phillips Screw (M3 x 6mm)</t>
   </si>
 </sst>
 </file>
@@ -645,7 +654,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="60.6328125" customWidth="1"/>
@@ -717,10 +726,10 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>22</v>
@@ -801,10 +810,10 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>33</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>10</v>
@@ -822,10 +831,10 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>34</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>10</v>
@@ -843,10 +852,10 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>10</v>
@@ -906,7 +915,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
-        <v>26</v>
+        <v>58</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>25</v>
@@ -927,10 +936,10 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
-        <v>27</v>
+        <v>57</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>24</v>
@@ -948,10 +957,10 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>24</v>
@@ -969,10 +978,10 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>24</v>
@@ -990,10 +999,10 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>24</v>
@@ -1011,10 +1020,12 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C18" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D18" s="2">
@@ -1030,10 +1041,10 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>24</v>
@@ -1051,10 +1062,10 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>24</v>
@@ -1072,10 +1083,12 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C21" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D21" s="2">
@@ -1091,113 +1104,132 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>22</v>
+        <v>56</v>
+      </c>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2" t="s">
+        <v>24</v>
       </c>
       <c r="D22" s="2">
         <v>1</v>
       </c>
       <c r="E22" s="3">
-        <v>9.19</v>
+        <v>4.57</v>
       </c>
       <c r="F22" s="3">
         <f>D22*E22</f>
-        <v>9.19</v>
+        <v>4.57</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B23" s="2"/>
-      <c r="C23" s="4"/>
+        <v>48</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>22</v>
+      </c>
       <c r="D23" s="2">
         <v>1</v>
       </c>
-      <c r="E23" s="3"/>
+      <c r="E23" s="3">
+        <v>9.19</v>
+      </c>
       <c r="F23" s="3">
-        <f t="shared" ref="F23:F26" si="1">D23*E23</f>
-        <v>0</v>
+        <f>D23*E23</f>
+        <v>9.19</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B24" s="2">
+        <v>49</v>
+      </c>
+      <c r="B24" s="2"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="2">
+        <v>1</v>
+      </c>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3">
+        <f t="shared" ref="F24:F27" si="1">D24*E24</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B25" s="2">
         <v>2337250</v>
       </c>
-      <c r="C24" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D24" s="2">
-        <v>1</v>
-      </c>
-      <c r="E24" s="3">
+      <c r="C25" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D25" s="2">
+        <v>1</v>
+      </c>
+      <c r="E25" s="3">
         <v>1.28</v>
       </c>
-      <c r="F24" s="3">
+      <c r="F25" s="3">
         <f t="shared" si="1"/>
         <v>1.28</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A25" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B25" s="2"/>
-      <c r="C25" s="4"/>
-      <c r="D25" s="2">
-        <v>1</v>
-      </c>
-      <c r="E25" s="3"/>
-      <c r="F25" s="3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B26" s="2"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="2">
+        <v>1</v>
+      </c>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A26" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="B26" s="2">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B27" s="2">
         <v>2010225</v>
       </c>
-      <c r="C26" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="D26" s="2">
-        <v>1</v>
-      </c>
-      <c r="E26" s="3">
+      <c r="C27" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D27" s="2">
+        <v>1</v>
+      </c>
+      <c r="E27" s="3">
         <v>1.19</v>
       </c>
-      <c r="F26" s="3">
+      <c r="F27" s="3">
         <f t="shared" si="1"/>
         <v>1.19</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A27" s="9" t="s">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B27" s="10"/>
-      <c r="C27" s="10"/>
-      <c r="D27" s="10"/>
-      <c r="E27" s="10"/>
-      <c r="F27" s="6">
-        <f>SUM(F2:F22)</f>
-        <v>420.44000000000023</v>
+      <c r="B28" s="10"/>
+      <c r="C28" s="10"/>
+      <c r="D28" s="10"/>
+      <c r="E28" s="10"/>
+      <c r="F28" s="6">
+        <f>SUM(F2:F23)</f>
+        <v>425.01000000000022</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A28:E28"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{7E1BCDF3-976F-4AEC-B6D9-914AB11C8929}"/>
@@ -1218,11 +1250,13 @@
     <hyperlink ref="C17" r:id="rId16" xr:uid="{54E91CA4-70D4-4C93-A3BC-A9525F2082F5}"/>
     <hyperlink ref="C19" r:id="rId17" xr:uid="{05371DE3-0E3D-4DFB-AB69-689437183BD1}"/>
     <hyperlink ref="C20" r:id="rId18" xr:uid="{CB12FF0B-0CD6-4EE9-BE97-CC2265FAA037}"/>
-    <hyperlink ref="C22" r:id="rId19" xr:uid="{D38EB2FB-A4F6-4217-AC04-0696B84A21B7}"/>
-    <hyperlink ref="C26" r:id="rId20" xr:uid="{552C1563-638D-45A1-AC3A-44E4E9AF22B2}"/>
-    <hyperlink ref="C24" r:id="rId21" xr:uid="{F9C09103-24AD-4BE0-98BE-EAA8979D84BF}"/>
+    <hyperlink ref="C23" r:id="rId19" xr:uid="{D38EB2FB-A4F6-4217-AC04-0696B84A21B7}"/>
+    <hyperlink ref="C27" r:id="rId20" xr:uid="{552C1563-638D-45A1-AC3A-44E4E9AF22B2}"/>
+    <hyperlink ref="C25" r:id="rId21" xr:uid="{F9C09103-24AD-4BE0-98BE-EAA8979D84BF}"/>
+    <hyperlink ref="C18" r:id="rId22" xr:uid="{CC0E5CCB-470C-4C72-9CD7-8E315F077547}"/>
+    <hyperlink ref="C21" r:id="rId23" xr:uid="{4243A696-8065-48E5-B878-C76DC0B860F0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId22"/>
+  <legacyDrawing r:id="rId24"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added a BOM link and updated price changes. Added a DrInfaredHeaterRemoteThermostat.csv for compatibility. ReadME was also read through and updated.
</commit_message>
<xml_diff>
--- a/ReadMeAssets/DrInfraredHeaterRemoteThermostat_BOM.xlsx
+++ b/ReadMeAssets/DrInfraredHeaterRemoteThermostat_BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\talyn\OneDrive\Desktop\Personel Projects\Shop Heater\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EDD81B0-2373-49EA-B874-4BDB67130E9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D299A2CA-0DF0-4BE0-872E-DE0F25F3DC3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-90" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="60">
   <si>
     <t>Description</t>
   </si>
@@ -237,6 +237,9 @@
   </si>
   <si>
     <t>Power Supply Phillips Screw (M3 x 6mm)</t>
+  </si>
+  <si>
+    <t>8251T3-8251T621</t>
   </si>
 </sst>
 </file>
@@ -864,11 +867,11 @@
         <v>3</v>
       </c>
       <c r="E10" s="3">
-        <v>1.22</v>
+        <v>1.26</v>
       </c>
       <c r="F10" s="3">
         <f t="shared" si="0"/>
-        <v>3.66</v>
+        <v>3.7800000000000002</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
@@ -1106,19 +1109,21 @@
       <c r="A22" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2" t="s">
+      <c r="B22" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D22" s="2">
         <v>1</v>
       </c>
       <c r="E22" s="3">
-        <v>4.57</v>
+        <v>5.28</v>
       </c>
       <c r="F22" s="3">
         <f>D22*E22</f>
-        <v>4.57</v>
+        <v>5.28</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
@@ -1135,11 +1140,11 @@
         <v>1</v>
       </c>
       <c r="E23" s="3">
-        <v>9.19</v>
+        <v>9.39</v>
       </c>
       <c r="F23" s="3">
         <f>D23*E23</f>
-        <v>9.19</v>
+        <v>9.39</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
@@ -1224,7 +1229,7 @@
       <c r="E28" s="10"/>
       <c r="F28" s="6">
         <f>SUM(F2:F23)</f>
-        <v>425.01000000000022</v>
+        <v>426.04000000000008</v>
       </c>
     </row>
   </sheetData>
@@ -1255,8 +1260,9 @@
     <hyperlink ref="C25" r:id="rId21" xr:uid="{F9C09103-24AD-4BE0-98BE-EAA8979D84BF}"/>
     <hyperlink ref="C18" r:id="rId22" xr:uid="{CC0E5CCB-470C-4C72-9CD7-8E315F077547}"/>
     <hyperlink ref="C21" r:id="rId23" xr:uid="{4243A696-8065-48E5-B878-C76DC0B860F0}"/>
+    <hyperlink ref="C22" r:id="rId24" xr:uid="{0878A9C1-11D5-409A-88D6-D158C3330B29}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId24"/>
+  <legacyDrawing r:id="rId25"/>
 </worksheet>
 </file>
</xml_diff>